<commit_message>
Maximum Sale is Found
</commit_message>
<xml_diff>
--- a/Day 2/Data_Analytics_Practice_Dataset.xlsx
+++ b/Day 2/Data_Analytics_Practice_Dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBABEE50-974E-451B-836D-1A9E2B6486F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC47816-B4BF-4CD5-9DB9-57F2AB69D053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38394,7 +38394,10 @@
       <c r="C49" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D49" s="3"/>
+      <c r="D49" s="3">
+        <f>MAX(I2:I41)</f>
+        <v>770000</v>
+      </c>
     </row>
     <row r="50" spans="3:4">
       <c r="C50" s="3" t="s">

</xml_diff>

<commit_message>
Minimum Sale is Found
</commit_message>
<xml_diff>
--- a/Day 2/Data_Analytics_Practice_Dataset.xlsx
+++ b/Day 2/Data_Analytics_Practice_Dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC47816-B4BF-4CD5-9DB9-57F2AB69D053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02CE30E-57AC-44F4-8028-AF70B526C68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38403,7 +38403,10 @@
       <c r="C50" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D50" s="3"/>
+      <c r="D50" s="3">
+        <f>MIN(I2:I41)</f>
+        <v>850</v>
+      </c>
     </row>
     <row r="51" spans="3:4">
       <c r="C51" s="3" t="s">

</xml_diff>

<commit_message>
Total Transaction is Counted
</commit_message>
<xml_diff>
--- a/Day 2/Data_Analytics_Practice_Dataset.xlsx
+++ b/Day 2/Data_Analytics_Practice_Dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02CE30E-57AC-44F4-8028-AF70B526C68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67614464-6181-45BA-9462-6B38E044EE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38412,7 +38412,10 @@
       <c r="C51" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D51" s="3"/>
+      <c r="D51" s="3">
+        <f>COUNT(I2:I41)</f>
+        <v>40</v>
+      </c>
     </row>
     <row r="52" spans="3:4">
       <c r="C52" s="3" t="s">

</xml_diff>

<commit_message>
Exployee Category is Found
</commit_message>
<xml_diff>
--- a/Day 2/Data_Analytics_Practice_Dataset.xlsx
+++ b/Day 2/Data_Analytics_Practice_Dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67614464-6181-45BA-9462-6B38E044EE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520A1944-FB15-4D32-BC9D-271FFB6493F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37116,7 +37116,10 @@
         <f>G2*H2</f>
         <v>220000</v>
       </c>
-      <c r="J2" s="3"/>
+      <c r="J2" s="3" t="str">
+        <f>IF(I2&gt;=500000,"Excellent",IF(I2&gt;=100000,"Better",IF(I2&gt;=80000,"Good","Grow")))</f>
+        <v>Better</v>
+      </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="7" t="s">
@@ -37148,7 +37151,10 @@
         <f t="shared" ref="I3:I41" si="1">G3*H3</f>
         <v>1200</v>
       </c>
-      <c r="J3" s="3"/>
+      <c r="J3" s="3" t="str">
+        <f t="shared" ref="J3:J41" si="2">IF(I3&gt;=500000,"Excellent",IF(I3&gt;=100000,"Better",IF(I3&gt;=80000,"Good","Grow")))</f>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="5" t="s">
@@ -37180,7 +37186,10 @@
         <f t="shared" si="1"/>
         <v>135000</v>
       </c>
-      <c r="J4" s="3"/>
+      <c r="J4" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="7" t="s">
@@ -37212,7 +37221,10 @@
         <f t="shared" si="1"/>
         <v>3600</v>
       </c>
-      <c r="J5" s="3"/>
+      <c r="J5" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="5" t="s">
@@ -37244,7 +37256,10 @@
         <f t="shared" si="1"/>
         <v>28000</v>
       </c>
-      <c r="J6" s="3"/>
+      <c r="J6" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="7" t="s">
@@ -37276,7 +37291,10 @@
         <f t="shared" si="1"/>
         <v>140000</v>
       </c>
-      <c r="J7" s="3"/>
+      <c r="J7" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="5" t="s">
@@ -37308,7 +37326,10 @@
         <f t="shared" si="1"/>
         <v>140000</v>
       </c>
-      <c r="J8" s="3"/>
+      <c r="J8" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="7" t="s">
@@ -37340,7 +37361,10 @@
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
-      <c r="J9" s="3"/>
+      <c r="J9" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="5" t="s">
@@ -37372,7 +37396,10 @@
         <f t="shared" si="1"/>
         <v>96000</v>
       </c>
-      <c r="J10" s="3"/>
+      <c r="J10" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Good</v>
+      </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="7" t="s">
@@ -37404,7 +37431,10 @@
         <f t="shared" si="1"/>
         <v>41800</v>
       </c>
-      <c r="J11" s="3"/>
+      <c r="J11" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="5" t="s">
@@ -37436,7 +37466,10 @@
         <f t="shared" si="1"/>
         <v>770000</v>
       </c>
-      <c r="J12" s="3"/>
+      <c r="J12" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Excellent</v>
+      </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="7" t="s">
@@ -37468,7 +37501,10 @@
         <f t="shared" si="1"/>
         <v>2400</v>
       </c>
-      <c r="J13" s="3"/>
+      <c r="J13" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="5" t="s">
@@ -37500,7 +37536,10 @@
         <f t="shared" si="1"/>
         <v>15000</v>
       </c>
-      <c r="J14" s="3"/>
+      <c r="J14" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="7" t="s">
@@ -37532,7 +37571,10 @@
         <f t="shared" si="1"/>
         <v>1350</v>
       </c>
-      <c r="J15" s="3"/>
+      <c r="J15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="5" t="s">
@@ -37564,7 +37606,10 @@
         <f t="shared" si="1"/>
         <v>24500</v>
       </c>
-      <c r="J16" s="3"/>
+      <c r="J16" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="7" t="s">
@@ -37596,7 +37641,10 @@
         <f t="shared" si="1"/>
         <v>76500</v>
       </c>
-      <c r="J17" s="3"/>
+      <c r="J17" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="5" t="s">
@@ -37628,7 +37676,10 @@
         <f t="shared" si="1"/>
         <v>17000</v>
       </c>
-      <c r="J18" s="3"/>
+      <c r="J18" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="7" t="s">
@@ -37660,7 +37711,10 @@
         <f t="shared" si="1"/>
         <v>32000</v>
       </c>
-      <c r="J19" s="3"/>
+      <c r="J19" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="5" t="s">
@@ -37692,7 +37746,10 @@
         <f t="shared" si="1"/>
         <v>39600</v>
       </c>
-      <c r="J20" s="3"/>
+      <c r="J20" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="7" t="s">
@@ -37724,7 +37781,10 @@
         <f t="shared" si="1"/>
         <v>385000</v>
       </c>
-      <c r="J21" s="3"/>
+      <c r="J21" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="5" t="s">
@@ -37756,7 +37816,10 @@
         <f t="shared" si="1"/>
         <v>385000</v>
       </c>
-      <c r="J22" s="3"/>
+      <c r="J22" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="7" t="s">
@@ -37788,7 +37851,10 @@
         <f t="shared" si="1"/>
         <v>21600</v>
       </c>
-      <c r="J23" s="3"/>
+      <c r="J23" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="5" t="s">
@@ -37820,7 +37886,10 @@
         <f t="shared" si="1"/>
         <v>210000</v>
       </c>
-      <c r="J24" s="3"/>
+      <c r="J24" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="7" t="s">
@@ -37852,7 +37921,10 @@
         <f t="shared" si="1"/>
         <v>52500</v>
       </c>
-      <c r="J25" s="3"/>
+      <c r="J25" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="5" t="s">
@@ -37884,7 +37956,10 @@
         <f t="shared" si="1"/>
         <v>532000</v>
       </c>
-      <c r="J26" s="3"/>
+      <c r="J26" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Excellent</v>
+      </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="7" t="s">
@@ -37916,7 +37991,10 @@
         <f t="shared" si="1"/>
         <v>40500</v>
       </c>
-      <c r="J27" s="3"/>
+      <c r="J27" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="5" t="s">
@@ -37948,7 +38026,10 @@
         <f t="shared" si="1"/>
         <v>850</v>
       </c>
-      <c r="J28" s="3"/>
+      <c r="J28" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="7" t="s">
@@ -37980,7 +38061,10 @@
         <f t="shared" si="1"/>
         <v>192000</v>
       </c>
-      <c r="J29" s="3"/>
+      <c r="J29" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="5" t="s">
@@ -38012,7 +38096,10 @@
         <f t="shared" si="1"/>
         <v>30800</v>
       </c>
-      <c r="J30" s="3"/>
+      <c r="J30" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="7" t="s">
@@ -38044,7 +38131,10 @@
         <f t="shared" si="1"/>
         <v>605000</v>
       </c>
-      <c r="J31" s="3"/>
+      <c r="J31" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Excellent</v>
+      </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="5" t="s">
@@ -38076,7 +38166,10 @@
         <f t="shared" si="1"/>
         <v>10800</v>
       </c>
-      <c r="J32" s="3"/>
+      <c r="J32" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="7" t="s">
@@ -38108,7 +38201,10 @@
         <f t="shared" si="1"/>
         <v>75000</v>
       </c>
-      <c r="J33" s="3"/>
+      <c r="J33" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="5" t="s">
@@ -38140,7 +38236,10 @@
         <f t="shared" si="1"/>
         <v>38500</v>
       </c>
-      <c r="J34" s="3"/>
+      <c r="J34" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="7" t="s">
@@ -38172,7 +38271,10 @@
         <f t="shared" si="1"/>
         <v>112000</v>
       </c>
-      <c r="J35" s="3"/>
+      <c r="J35" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="5" t="s">
@@ -38204,7 +38306,10 @@
         <f t="shared" si="1"/>
         <v>112000</v>
       </c>
-      <c r="J36" s="3"/>
+      <c r="J36" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="7" t="s">
@@ -38236,7 +38341,10 @@
         <f t="shared" si="1"/>
         <v>13500</v>
       </c>
-      <c r="J37" s="3"/>
+      <c r="J37" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="5" t="s">
@@ -38268,7 +38376,10 @@
         <f t="shared" si="1"/>
         <v>11050</v>
       </c>
-      <c r="J38" s="3"/>
+      <c r="J38" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="7" t="s">
@@ -38300,7 +38411,10 @@
         <f t="shared" si="1"/>
         <v>128000</v>
       </c>
-      <c r="J39" s="3"/>
+      <c r="J39" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Better</v>
+      </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="5" t="s">
@@ -38332,7 +38446,10 @@
         <f t="shared" si="1"/>
         <v>26400</v>
       </c>
-      <c r="J40" s="3"/>
+      <c r="J40" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Grow</v>
+      </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="7" t="s">
@@ -38364,7 +38481,10 @@
         <f t="shared" si="1"/>
         <v>660000</v>
       </c>
-      <c r="J41" s="3"/>
+      <c r="J41" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Excellent</v>
+      </c>
     </row>
     <row r="46" spans="1:10" ht="15" customHeight="1">
       <c r="C46" s="9" t="s">

</xml_diff>

<commit_message>
Number of Execellent Emplyoee is Found
</commit_message>
<xml_diff>
--- a/Day 2/Data_Analytics_Practice_Dataset.xlsx
+++ b/Day 2/Data_Analytics_Practice_Dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520A1944-FB15-4D32-BC9D-271FFB6493F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22206CB4-5A20-497C-81FC-8B528DC39A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38541,7 +38541,10 @@
       <c r="C52" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D52" s="3"/>
+      <c r="D52" s="3">
+        <f>COUNTIF(J2:J41,"Excellent")</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="53" spans="3:4">
       <c r="C53" s="3" t="s">

</xml_diff>

<commit_message>
Number of Good Emplyoee is Found
</commit_message>
<xml_diff>
--- a/Day 2/Data_Analytics_Practice_Dataset.xlsx
+++ b/Day 2/Data_Analytics_Practice_Dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22206CB4-5A20-497C-81FC-8B528DC39A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37B8BC47-2DDA-4F66-BECF-350E24787A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38550,7 +38550,10 @@
       <c r="C53" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D53" s="3"/>
+      <c r="D53" s="3">
+        <f>COUNTIF(J2:J41,"Good")</f>
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>